<commit_message>
John en Leon nemen ze over yay
</commit_message>
<xml_diff>
--- a/Takenrooster 01-10-26.xlsx
+++ b/Takenrooster 01-10-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\.Code\Volleybal\message_builder\message_builder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\.Code\message_builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F559356-A7FC-49D3-AB62-DBFC13665ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF604DB7-61F9-4917-8650-ABAE474AB52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="thuiswedstrijden" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1487" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1490" uniqueCount="326">
   <si>
     <t>vnr</t>
   </si>
@@ -1273,14 +1273,14 @@
       <font>
         <color theme="1"/>
       </font>
-      <numFmt numFmtId="166" formatCode="h:mm"/>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
         <color theme="1"/>
       </font>
-      <numFmt numFmtId="166" formatCode="h:mm"/>
+      <numFmt numFmtId="25" formatCode="h:mm"/>
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -4236,7 +4236,9 @@
         <v>28</v>
       </c>
       <c r="Q46" s="29"/>
-      <c r="R46" s="29"/>
+      <c r="R46" s="29" t="s">
+        <v>322</v>
+      </c>
       <c r="S46" s="17"/>
       <c r="T46" s="17" t="s">
         <v>106</v>
@@ -4450,7 +4452,9 @@
         <v>28</v>
       </c>
       <c r="Q50" s="29"/>
-      <c r="R50" s="29"/>
+      <c r="R50" s="29" t="s">
+        <v>324</v>
+      </c>
       <c r="S50" s="17"/>
       <c r="T50" s="17" t="s">
         <v>106</v>
@@ -4556,7 +4560,9 @@
         <v>28</v>
       </c>
       <c r="Q52" s="29"/>
-      <c r="R52" s="29"/>
+      <c r="R52" s="29" t="s">
+        <v>322</v>
+      </c>
       <c r="S52" s="17"/>
       <c r="T52" s="17" t="s">
         <v>106</v>

</xml_diff>